<commit_message>
Fix builtin time format locale (#744)
* Add locale-sensitive GetNumberFormatString for built-in time formats 20 and 21

Extend GetBuiltinNumberFormat(numFmtId, provider) to derive format strings
for built-in indices 20 (h:mm) and 21 (h:mm:ss) from the provider's
ShortTimePattern and LongTimePattern respectively, consistent with how
index 22 already derives its time component.

Also update Issue461.xlsx to include cells with numFmtId 20 and 21,
and add corresponding tests.

* Fix GetNumberFormatString for indices 20/21: fall back to spec string on 12h locales

Indices 20 (h:mm) and 21 (h:mm:ss) are explicitly non-AM/PM formats.
On 12h locales like en-US, deriving from ShortTimePattern/LongTimePattern
would incorrectly add AM/PM. Fall back to the hardcoded spec string when
the derived pattern contains AM/PM or A/P.
</commit_message>
<xml_diff>
--- a/src/TestData/Issue461.xlsx
+++ b/src/TestData/Issue461.xlsx
@@ -35,12 +35,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
 </styleSheet>
 </file>
@@ -61,6 +63,12 @@
       <c r="D1" s="4">
         <v>44927</v>
       </c>
+      <c r="E1" s="5">
+        <v>44927</v>
+      </c>
+      <c r="F1" s="6">
+        <v>44927</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>